<commit_message>
Expand Sugar News retrieval and validation
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-02.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-02.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,37 +505,105 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="114.75" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>印度食糖出口禁令继续影响南亚节前贸易流向，尼泊尔市场出现走私增加的报道。正规出口受限会减少周边市场可获得糖源，并使节前补库需求转向非正规渠道，从而支撑区域糖价。来源：The Kathmandu Post（https://news.google.com/rss/articles/CBMiwgFBVV95cUxNUndBMUo1U2xfdXk4UHRMNThHOWM5bnRBNWVyQjdnVExhRWRzTVRObENoYWpvdTcwQzE4YTR0eVZtQklGNjhGMWpRMHp2OThmN3VDN0c2VjdRRkk0LU93eFpKU2dDRUU0Mjl4OV82b0ZrdW45RnpGcFd5UmVrQVBOSldIOExLTHBXZGZVSWJXQ0tyNDE3c3VRbWdsUjRwaTB4Z280VEdoMm5ZQ2U0SFI0RXd0bG9UdHJ0S0JkaEEyOHpQZw?oc=5）</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>利多：出口禁令限制印度正规糖源外流，节前需求转向非正规贸易会加剧周边市场供应紧张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="180" customHeight="1" s="2">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>印度中央政府促成糖厂以Rs 4263销售PDM，交易主体为印度糖厂。副产品销售变现有助于改善糖厂现金流和运营稳定性，降低压榨季资金压力。来源：AgroSpectrum India（https://news.google.com/rss/articles/CBMizwFBVV95cUxONUlzdEJuZWVCVUUzRmNmNzNvei1VanJoNk9uQnpVa0tXdllEQ2dQOEVNay0xUHI2d2g0bjJSZUhhZVBHR3p2VVJ4dHBjZi04MGRzNnNuMHNjM094Y0l5WnM0d25KUVBIcTBpek9GSnpDdjBIa05RWGlzcGE5dU5RamE5WERTMEZEUTVxcjU5RTU3NFJuRW9MYzEwZmpCQ2NLS3NiQUs3RXEtNVNGVGNKTGp4Y2EzM182OHVtQmlrRm41NnlNOTItX2wxNDVyVVE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>利空：糖厂副产品销售价格明确有助于改善现金流，间接支持压榨和制糖经营稳定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="180" customHeight="1" s="2">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>印度政府称，如果没有乙醇掺混，汽油价格可能达到每升Rs 125。乙醇掺混降低燃料成本的同时扩大乙醇需求，糖厂将更多甘蔗、糖蜜或糖浆转向制醇时，食糖供应预期会受到支撑。来源：The Economic Times（https://news.google.com/rss/articles/CBMi3AFBVV95cUxPdlUtbm9TX0daQ05EeXlFazBoWEltNUFrRFgtNlFBbU5hUVdjcEhwUFcxN0xHRm9CMUlOcnV3MzUzQVBHMXRtRHg2OVI0d2VFWEQ5Q0t0eTRDZ0l6c09fN0lhbHItZmpQN1hnQkNqMmliR0Y1OXp4UkIxclhqVm1vdG02TTdmbXB4VU5mN1pONHRPQ0R0OUYyYzlfeTZ5VnBjOHdhRmZ5SEtqdDFRY2luNkE5ZUNrTmNXQmNRME5Ja1ZoV09mcWE4Vm9DQVFoU0swQ2hvcjU0dU9LNVZW0gHiAUFVX3lxTE9aeUtJTHlUd3lLamxJeTVRNzAxaW51Skx5MjVKSFk4SFNwV0YzMWpZZnZVd2F5UnFmUXNLM2ppalZrSWZuT2JZS0pWTUdxZE1tOEFfLU5MWHl1RjktT3FCQzZ4MzFfYkFxeElKbU0yN3BpWGdfbnNONWNzR2V2c2xoSHZTNEtJWlFfbFJvNDJjUHFCMUJOM3ljMHdrbC13Sjk5TFJwRV8yLUpJVTJ2dHhXQ3BjMWphcWZVamdIdXNfbjVVakZfWnc1Y2NPN0J3b2NfTU9Wc0xvNFZiZ1F3NnlCTXc?oc=5）</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>利多：乙醇掺混扩大燃料端需求，会增强甘蔗、糖蜜和糖浆制醇吸引力，减少部分制糖供应。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="114.75" customHeight="1" s="2">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
           <t>泰国</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>泰国气象局预报（2026-08-02），乌隆他尼、黎府、那空沙旺、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="118.05" customHeight="1" s="2">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="6" ht="118.05" customHeight="1" s="2">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>中国</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="180" customHeight="1" s="2">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>菲律宾棉兰老岛蔗农组织预警，甘蔗病虫害已扩散至4 provinces。病虫害扩大将影响甘蔗生长和可收获糖料，若防控不及时，后续食糖产量预期会下调。来源：Inquirer.net（https://news.google.com/rss/articles/CBMirAFBVV95cUxQeWN2OWhuejVsRDFEZDVsUHc3Z0YwZHlNWmVpY1JaWV9LczFtb0tvUDFMVzJLVVJZa3M0Ml8zSWMxRUFYMkxSUV94SjRFa1lCQjZqYlF2dnA4ZF9mS2dRVV9kbXNHXzhKRnBqMkEtR1FadWlZVzhvZFRyODBhRXdxdFpYVlhmSElVYkJadm5PeHhZQjFiMVRBXzBKTTBWVl9CSnhISTFhX1dGNGcy0gGyAUFVX3lxTE9XdVdFQ3JWWEFicjRCYWlBSHRGTnVmUk4zS0xIWlJHdE9RaHdBbENqcnVxZGs5aGpjekV1RC1DYkJxVXprUVphd1dqR2t0ckVqdHh1NFZVV3lfZFAzc3BUa3ptcmdsMDJ3WHhRWVQ4ZUVuVkdXc0V1TkhneEpZUFN4U1NGOFVyR040dTZsTGQyejRVbXpYS0FXUHNWY3FzN0M4c1dpYXRNLUtMU1pQbWVFdkE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>利多：病虫害扩散会压低甘蔗单产并削弱糖料供应稳定性，从而支撑糖价。</t>
         </is>
       </c>
     </row>

</xml_diff>